<commit_message>
Add random spot-check validation and update ENSDF data
Introduced random spot-check validation guidelines to chatmode, copilot instructions, and image extraction prompt for improved data quality assurance. Updated ENSDF file for 35Cl (1972HU10): added missing gamma transitions, restructured resonance comments, and removed redundant resonance comment lines for clarity and compliance.
</commit_message>
<xml_diff>
--- a/A35/Cl35/temp/34Spg35Cl.xlsx
+++ b/A35/Cl35/temp/34Spg35Cl.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\A35\Cl35\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5372CE7-3DCC-4820-A387-38ED9D019AFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAECE17A-76D3-4868-9DED-C8CA5B392324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="5" xr2:uid="{C580B2C4-D120-4EC4-942B-ED4733C9AE26}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="6" xr2:uid="{C580B2C4-D120-4EC4-942B-ED4733C9AE26}"/>
   </bookViews>
   <sheets>
     <sheet name="1976SP08_Ep" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,8 @@
     <sheet name="1976ME12_R" sheetId="4" r:id="rId3"/>
     <sheet name="1976ME12_B" sheetId="5" r:id="rId4"/>
     <sheet name="1973FA07" sheetId="6" r:id="rId5"/>
-    <sheet name="1972HU10" sheetId="7" r:id="rId6"/>
+    <sheet name="1972HU10_R" sheetId="7" r:id="rId6"/>
+    <sheet name="1972HU10_B" sheetId="9" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="384">
   <si>
     <t>No.</t>
   </si>
@@ -1090,6 +1091,123 @@
   </si>
   <si>
     <t>Exi_original</t>
+  </si>
+  <si>
+    <t>Red: Resonances without γ</t>
+  </si>
+  <si>
+    <t>≤0.2</t>
+  </si>
+  <si>
+    <t>≤5</t>
+  </si>
+  <si>
+    <t>≤1</t>
+  </si>
+  <si>
+    <t>≤3</t>
+  </si>
+  <si>
+    <t>92±1</t>
+  </si>
+  <si>
+    <t>8±1</t>
+  </si>
+  <si>
+    <t>81±3</t>
+  </si>
+  <si>
+    <t>13±2</t>
+  </si>
+  <si>
+    <t>89±2</t>
+  </si>
+  <si>
+    <t>11±2</t>
+  </si>
+  <si>
+    <t>83±3</t>
+  </si>
+  <si>
+    <t>17±3</t>
+  </si>
+  <si>
+    <t>93±3</t>
+  </si>
+  <si>
+    <t>7±3</t>
+  </si>
+  <si>
+    <t>21±3</t>
+  </si>
+  <si>
+    <t>74±5</t>
+  </si>
+  <si>
+    <t>5±3</t>
+  </si>
+  <si>
+    <t>97±2</t>
+  </si>
+  <si>
+    <t>3±2</t>
+  </si>
+  <si>
+    <t>50±20</t>
+  </si>
+  <si>
+    <t>18±6</t>
+  </si>
+  <si>
+    <t>27±8</t>
+  </si>
+  <si>
+    <t>62±6</t>
+  </si>
+  <si>
+    <t>31±5</t>
+  </si>
+  <si>
+    <t>7±2</t>
+  </si>
+  <si>
+    <t>70±5</t>
+  </si>
+  <si>
+    <t>53±10</t>
+  </si>
+  <si>
+    <t>47±10</t>
+  </si>
+  <si>
+    <t>70±10</t>
+  </si>
+  <si>
+    <t>10±5</t>
+  </si>
+  <si>
+    <t>40±20</t>
+  </si>
+  <si>
+    <t>25±10</t>
+  </si>
+  <si>
+    <t>60±20</t>
+  </si>
+  <si>
+    <t>80±10</t>
+  </si>
+  <si>
+    <t>20±10</t>
+  </si>
+  <si>
+    <t>Initial Level Ex_keV</t>
+  </si>
+  <si>
+    <t>Unknown final levels</t>
+  </si>
+  <si>
+    <t>≤ 0.2</t>
   </si>
 </sst>
 </file>
@@ -1100,7 +1218,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0_);\(0.0\)"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1144,6 +1262,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1165,7 +1295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1273,6 +1403,15 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -11105,7 +11244,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23EB2F7C-C222-4E6A-976F-47714D7661A7}">
-  <dimension ref="A1:AD61"/>
+  <dimension ref="A1:AD63"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="23"/>
@@ -11246,6 +11385,7 @@
       <c r="I3" s="23" t="s">
         <v>300</v>
       </c>
+      <c r="J3" s="13"/>
       <c r="K3" s="13" t="s">
         <v>342</v>
       </c>
@@ -11301,6 +11441,7 @@
       <c r="I4" s="23">
         <v>0.5</v>
       </c>
+      <c r="J4" s="30"/>
       <c r="K4" s="28">
         <f>L4/35*34+$A$1</f>
         <v>7066.3428571428576</v>
@@ -11373,6 +11514,7 @@
       <c r="I5" s="23">
         <v>0.5</v>
       </c>
+      <c r="J5" s="30"/>
       <c r="K5" s="28">
         <f t="shared" ref="K5:K51" si="3">L5/35*34+$A$1</f>
         <v>7103.2571428571428</v>
@@ -11441,6 +11583,7 @@
       <c r="I6" s="23">
         <v>0.5</v>
       </c>
+      <c r="J6" s="30"/>
       <c r="K6" s="28">
         <f t="shared" si="3"/>
         <v>7179.0285714285719</v>
@@ -11511,6 +11654,7 @@
       <c r="I7" s="23">
         <v>0.3</v>
       </c>
+      <c r="J7" s="30"/>
       <c r="K7" s="28">
         <f t="shared" si="3"/>
         <v>7194.5714285714284</v>
@@ -11579,6 +11723,7 @@
       <c r="I8" s="23">
         <v>0.7</v>
       </c>
+      <c r="J8" s="30"/>
       <c r="K8" s="28">
         <f t="shared" si="3"/>
         <v>7226.6285714285714</v>
@@ -11649,6 +11794,7 @@
       <c r="I9" s="23">
         <v>0.5</v>
       </c>
+      <c r="J9" s="30"/>
       <c r="K9" s="28">
         <f t="shared" si="3"/>
         <v>7234.4</v>
@@ -11715,6 +11861,7 @@
       <c r="I10" s="23">
         <v>0.6</v>
       </c>
+      <c r="J10" s="30"/>
       <c r="K10" s="28">
         <f t="shared" si="3"/>
         <v>7272.2857142857147</v>
@@ -11785,6 +11932,7 @@
       <c r="I11" s="23">
         <v>0.9</v>
       </c>
+      <c r="J11" s="30"/>
       <c r="K11" s="28">
         <f t="shared" si="3"/>
         <v>7361.6571428571433</v>
@@ -11859,6 +12007,7 @@
       <c r="I12" s="23">
         <v>0.6</v>
       </c>
+      <c r="J12" s="30"/>
       <c r="K12" s="28">
         <f t="shared" si="3"/>
         <v>7395.6571428571433</v>
@@ -11927,6 +12076,7 @@
       <c r="I13" s="23">
         <v>0.8</v>
       </c>
+      <c r="J13" s="30"/>
       <c r="K13" s="28">
         <f t="shared" si="3"/>
         <v>7451.0285714285719</v>
@@ -11990,7 +12140,8 @@
       <c r="I14" s="23">
         <v>3</v>
       </c>
-      <c r="K14" s="28">
+      <c r="J14" s="32"/>
+      <c r="K14" s="21">
         <f t="shared" si="3"/>
         <v>7502.5142857142855</v>
       </c>
@@ -12054,7 +12205,8 @@
       <c r="I15" s="23">
         <v>0.6</v>
       </c>
-      <c r="K15" s="28">
+      <c r="J15" s="32"/>
+      <c r="K15" s="21">
         <f t="shared" si="3"/>
         <v>7503.4857142857145</v>
       </c>
@@ -12115,6 +12267,7 @@
       <c r="I16" s="23">
         <v>0.9</v>
       </c>
+      <c r="J16" s="30"/>
       <c r="K16" s="28">
         <f t="shared" si="3"/>
         <v>7520</v>
@@ -12181,6 +12334,7 @@
       <c r="I17" s="23">
         <v>0.8</v>
       </c>
+      <c r="J17" s="30"/>
       <c r="K17" s="28">
         <f t="shared" si="3"/>
         <v>7550.1142857142859</v>
@@ -12249,6 +12403,7 @@
       <c r="I18" s="23">
         <v>5</v>
       </c>
+      <c r="J18" s="30"/>
       <c r="K18" s="28">
         <f t="shared" si="3"/>
         <v>7561.7714285714292</v>
@@ -12317,6 +12472,7 @@
       <c r="I19" s="23">
         <v>1.2</v>
       </c>
+      <c r="J19" s="30"/>
       <c r="K19" s="28">
         <f t="shared" si="3"/>
         <v>7601.6</v>
@@ -12390,11 +12546,12 @@
         <v>0.5</v>
       </c>
       <c r="H20" s="23">
-        <v>48384</v>
+        <v>4838</v>
       </c>
       <c r="I20" s="23">
         <v>3</v>
       </c>
+      <c r="J20" s="30"/>
       <c r="K20" s="28">
         <f t="shared" si="3"/>
         <v>7619.0857142857149</v>
@@ -12463,6 +12620,7 @@
       <c r="I21" s="23">
         <v>2</v>
       </c>
+      <c r="J21" s="30"/>
       <c r="K21" s="28">
         <f t="shared" si="3"/>
         <v>7656.971428571429</v>
@@ -12529,6 +12687,7 @@
       <c r="I22" s="23">
         <v>1</v>
       </c>
+      <c r="J22" s="30"/>
       <c r="K22" s="28">
         <f t="shared" si="3"/>
         <v>7672.5142857142855</v>
@@ -12599,6 +12758,7 @@
       <c r="I23" s="23">
         <v>5</v>
       </c>
+      <c r="J23" s="30"/>
       <c r="K23" s="28">
         <f t="shared" si="3"/>
         <v>7686.1142857142859</v>
@@ -12669,6 +12829,7 @@
       <c r="I24" s="23">
         <v>5</v>
       </c>
+      <c r="J24" s="30"/>
       <c r="K24" s="28">
         <f t="shared" si="3"/>
         <v>7693.8857142857141</v>
@@ -12733,6 +12894,7 @@
       <c r="I25" s="23">
         <v>3</v>
       </c>
+      <c r="J25" s="30"/>
       <c r="K25" s="28">
         <f t="shared" si="3"/>
         <v>7707.4857142857145</v>
@@ -12801,6 +12963,7 @@
       <c r="I26" s="23">
         <v>5</v>
       </c>
+      <c r="J26" s="30"/>
       <c r="K26" s="28">
         <f t="shared" si="3"/>
         <v>7746.3428571428576</v>
@@ -12869,6 +13032,7 @@
       <c r="I27" s="23">
         <v>3</v>
       </c>
+      <c r="J27" s="33"/>
       <c r="K27" s="28">
         <f t="shared" si="3"/>
         <v>7778.4</v>
@@ -12941,6 +13105,7 @@
       <c r="I28" s="23">
         <v>3</v>
       </c>
+      <c r="J28" s="33"/>
       <c r="K28" s="28">
         <f t="shared" si="3"/>
         <v>7783.2571428571428</v>
@@ -13008,6 +13173,7 @@
       <c r="I29" s="23">
         <v>3</v>
       </c>
+      <c r="J29" s="33"/>
       <c r="K29" s="28">
         <f t="shared" si="3"/>
         <v>7798.8</v>
@@ -13068,6 +13234,7 @@
       <c r="I30" s="23">
         <v>3</v>
       </c>
+      <c r="J30" s="33"/>
       <c r="K30" s="28">
         <f t="shared" si="3"/>
         <v>7840.5714285714284</v>
@@ -13136,6 +13303,7 @@
       <c r="I31" s="23">
         <v>5</v>
       </c>
+      <c r="J31" s="33"/>
       <c r="K31" s="28">
         <f t="shared" si="3"/>
         <v>7868.7428571428572</v>
@@ -13200,6 +13368,7 @@
       <c r="I32" s="23">
         <v>5</v>
       </c>
+      <c r="J32" s="33"/>
       <c r="K32" s="28">
         <f t="shared" si="3"/>
         <v>7881.3714285714286</v>
@@ -13270,6 +13439,7 @@
       <c r="I33" s="23">
         <v>5</v>
       </c>
+      <c r="J33" s="33"/>
       <c r="K33" s="28">
         <f t="shared" si="3"/>
         <v>7899.8285714285712</v>
@@ -13336,6 +13506,7 @@
       <c r="I34" s="23">
         <v>3</v>
       </c>
+      <c r="J34" s="33"/>
       <c r="K34" s="28">
         <f t="shared" si="3"/>
         <v>7924.1142857142859</v>
@@ -13408,6 +13579,7 @@
       <c r="I35" s="23">
         <v>5</v>
       </c>
+      <c r="J35" s="33"/>
       <c r="K35" s="28">
         <f t="shared" si="3"/>
         <v>7970.7428571428572</v>
@@ -13470,6 +13642,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J36" s="33"/>
       <c r="K36" s="28">
         <f t="shared" si="3"/>
         <v>7988.2285714285717</v>
@@ -13524,6 +13697,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J37" s="33"/>
       <c r="K37" s="28">
         <f t="shared" si="3"/>
         <v>7996.971428571429</v>
@@ -13582,6 +13756,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J38" s="33"/>
       <c r="K38" s="28">
         <f t="shared" si="3"/>
         <v>8002.8</v>
@@ -13642,6 +13817,7 @@
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
+      <c r="J39" s="33"/>
       <c r="K39" s="28">
         <f t="shared" si="3"/>
         <v>8006.6857142857143</v>
@@ -13698,6 +13874,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J40" s="33"/>
       <c r="K40" s="28">
         <f t="shared" si="3"/>
         <v>8035.8285714285712</v>
@@ -13760,6 +13937,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J41" s="33"/>
       <c r="K41" s="28">
         <f t="shared" si="3"/>
         <v>8039.7142857142862</v>
@@ -13820,6 +13998,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J42" s="33"/>
       <c r="K42" s="28">
         <f t="shared" si="3"/>
         <v>8076.6285714285714</v>
@@ -13880,6 +14059,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J43" s="33"/>
       <c r="K43" s="28">
         <f t="shared" si="3"/>
         <v>8097.0285714285719</v>
@@ -13944,6 +14124,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J44" s="33"/>
       <c r="K44" s="28">
         <f t="shared" si="3"/>
         <v>8107.7142857142862</v>
@@ -14010,6 +14191,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J45" s="33"/>
       <c r="K45" s="28">
         <f t="shared" si="3"/>
         <v>8114.5142857142855</v>
@@ -14072,6 +14254,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J46" s="33"/>
       <c r="K46" s="28">
         <f t="shared" si="3"/>
         <v>8147.5428571428574</v>
@@ -14136,6 +14319,7 @@
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
+      <c r="J47" s="33"/>
       <c r="K47" s="28">
         <f t="shared" si="3"/>
         <v>8157.2571428571428</v>
@@ -14198,6 +14382,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J48" s="33"/>
       <c r="K48" s="28">
         <f t="shared" si="3"/>
         <v>8180.5714285714284</v>
@@ -14258,6 +14443,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J49" s="33"/>
       <c r="K49" s="28">
         <f t="shared" si="3"/>
         <v>8209.7142857142862</v>
@@ -14299,7 +14485,7 @@
       <c r="AB49" s="27"/>
     </row>
     <row r="50" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A50" s="12">
+      <c r="A50" s="40">
         <f t="shared" si="0"/>
         <v>8243.908571428572</v>
       </c>
@@ -14320,6 +14506,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J50" s="34"/>
       <c r="K50" s="28">
         <f t="shared" si="3"/>
         <v>8218.4571428571435</v>
@@ -14355,7 +14542,7 @@
       <c r="AB50" s="35"/>
     </row>
     <row r="51" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A51" s="12">
+      <c r="A51" s="40">
         <f t="shared" si="0"/>
         <v>8270.8171428571441</v>
       </c>
@@ -14376,6 +14563,7 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="J51" s="27"/>
       <c r="K51" s="28">
         <f t="shared" si="3"/>
         <v>8384.5714285714294</v>
@@ -14417,7 +14605,7 @@
       <c r="AB51" s="27"/>
     </row>
     <row r="52" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A52" s="12">
+      <c r="A52" s="40">
         <f t="shared" si="0"/>
         <v>8278.7828571428581</v>
       </c>
@@ -14444,11 +14632,11 @@
       </c>
       <c r="O52" s="7"/>
       <c r="P52" s="7">
-        <f t="shared" ref="O52:AA52" si="5">$M51-P2</f>
+        <f>$M51-P2</f>
         <v>6619.2</v>
       </c>
       <c r="Q52" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="P52:Y52" si="5">$M51-Q2</f>
         <v>5736.4</v>
       </c>
       <c r="R52" s="7">
@@ -14475,7 +14663,7 @@
       <c r="AA52" s="7"/>
     </row>
     <row r="53" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A53" s="12">
+      <c r="A53" s="40">
         <f t="shared" si="0"/>
         <v>8284.5142857142855</v>
       </c>
@@ -14498,7 +14686,7 @@
       </c>
     </row>
     <row r="54" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A54" s="12">
+      <c r="A54" s="40">
         <f t="shared" si="0"/>
         <v>8289.954285714286</v>
       </c>
@@ -14521,7 +14709,7 @@
       </c>
     </row>
     <row r="55" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A55" s="12">
+      <c r="A55" s="40">
         <f t="shared" si="0"/>
         <v>8300.057142857142</v>
       </c>
@@ -14544,7 +14732,7 @@
       </c>
     </row>
     <row r="56" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A56" s="12">
+      <c r="A56" s="40">
         <f t="shared" si="0"/>
         <v>8320.1657142857148</v>
       </c>
@@ -14567,7 +14755,7 @@
       </c>
     </row>
     <row r="57" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A57" s="12">
+      <c r="A57" s="40">
         <f t="shared" si="0"/>
         <v>8323.8571428571431</v>
       </c>
@@ -14613,7 +14801,7 @@
       </c>
     </row>
     <row r="59" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A59" s="12">
+      <c r="A59" s="40">
         <f t="shared" si="0"/>
         <v>8391.3714285714286</v>
       </c>
@@ -14636,7 +14824,7 @@
       </c>
     </row>
     <row r="60" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A60" s="12">
+      <c r="A60" s="40">
         <f t="shared" si="0"/>
         <v>8407.4971428571425</v>
       </c>
@@ -14659,7 +14847,7 @@
       </c>
     </row>
     <row r="61" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A61" s="12">
+      <c r="A61" s="40">
         <f t="shared" si="0"/>
         <v>8411.7714285714283</v>
       </c>
@@ -14679,6 +14867,11 @@
       <c r="F61" s="25">
         <f t="shared" si="2"/>
         <v>0.3</v>
+      </c>
+    </row>
+    <row r="63" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A63" s="41" t="s">
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -14686,4 +14879,624 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D8AF1C-2651-4BD5-9C4B-97413D66179F}">
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="42" t="s">
+        <v>381</v>
+      </c>
+      <c r="B1" s="42">
+        <v>0</v>
+      </c>
+      <c r="C1" s="42">
+        <v>1219.0999999999999</v>
+      </c>
+      <c r="D1" s="42">
+        <v>1762.8</v>
+      </c>
+      <c r="E1" s="42">
+        <v>2645.6</v>
+      </c>
+      <c r="F1" s="42">
+        <v>2694</v>
+      </c>
+      <c r="G1" s="42">
+        <v>3002.7</v>
+      </c>
+      <c r="H1" s="42">
+        <v>3162.5</v>
+      </c>
+      <c r="I1" s="42">
+        <v>4177.2</v>
+      </c>
+      <c r="J1" s="42" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="42">
+        <v>1219.0999999999999</v>
+      </c>
+      <c r="B2" s="42">
+        <v>100</v>
+      </c>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="42">
+        <v>1762.8</v>
+      </c>
+      <c r="B3" s="42">
+        <v>100</v>
+      </c>
+      <c r="C3" s="42" t="s">
+        <v>346</v>
+      </c>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="42">
+        <v>2645.6</v>
+      </c>
+      <c r="B4" s="42" t="s">
+        <v>350</v>
+      </c>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42" t="s">
+        <v>351</v>
+      </c>
+      <c r="E4" s="42"/>
+      <c r="F4" s="42"/>
+      <c r="G4" s="42"/>
+      <c r="H4" s="42"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="42"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="42">
+        <v>2694</v>
+      </c>
+      <c r="B5" s="42" t="s">
+        <v>352</v>
+      </c>
+      <c r="C5" s="42" t="s">
+        <v>268</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>353</v>
+      </c>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
+      <c r="J5" s="42"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="42">
+        <v>3002.7</v>
+      </c>
+      <c r="B6" s="42">
+        <v>100</v>
+      </c>
+      <c r="C6" s="42" t="s">
+        <v>347</v>
+      </c>
+      <c r="D6" s="42" t="s">
+        <v>348</v>
+      </c>
+      <c r="E6" s="42"/>
+      <c r="F6" s="42"/>
+      <c r="G6" s="42"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="42">
+        <v>3162.5</v>
+      </c>
+      <c r="B7" s="42" t="s">
+        <v>354</v>
+      </c>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42" t="s">
+        <v>383</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>355</v>
+      </c>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="42"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="42">
+        <v>3917.9</v>
+      </c>
+      <c r="B8" s="42" t="s">
+        <v>356</v>
+      </c>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42" t="s">
+        <v>357</v>
+      </c>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="42"/>
+      <c r="J8" s="42"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="42">
+        <v>3942.6</v>
+      </c>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42" t="s">
+        <v>358</v>
+      </c>
+      <c r="E9" s="42" t="s">
+        <v>359</v>
+      </c>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="42"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="42">
+        <v>3967.3</v>
+      </c>
+      <c r="B10" s="42" t="s">
+        <v>360</v>
+      </c>
+      <c r="C10" s="42" t="s">
+        <v>361</v>
+      </c>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="42" t="s">
+        <v>362</v>
+      </c>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="42"/>
+      <c r="J10" s="42"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="42">
+        <v>4058.4</v>
+      </c>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42" t="s">
+        <v>363</v>
+      </c>
+      <c r="D11" s="42" t="s">
+        <v>364</v>
+      </c>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
+      <c r="H11" s="42"/>
+      <c r="I11" s="42"/>
+      <c r="J11" s="42"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="42">
+        <v>4111</v>
+      </c>
+      <c r="B12" s="42" t="s">
+        <v>365</v>
+      </c>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42" t="s">
+        <v>365</v>
+      </c>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
+      <c r="H12" s="42"/>
+      <c r="I12" s="42"/>
+      <c r="J12" s="42"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="42">
+        <v>4173</v>
+      </c>
+      <c r="B13" s="42" t="s">
+        <v>263</v>
+      </c>
+      <c r="C13" s="42" t="s">
+        <v>349</v>
+      </c>
+      <c r="D13" s="42" t="s">
+        <v>366</v>
+      </c>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42" t="s">
+        <v>367</v>
+      </c>
+      <c r="G13" s="42"/>
+      <c r="H13" s="42"/>
+      <c r="I13" s="42"/>
+      <c r="J13" s="42"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="42">
+        <v>4177.2</v>
+      </c>
+      <c r="B14" s="42" t="s">
+        <v>368</v>
+      </c>
+      <c r="C14" s="42" t="s">
+        <v>369</v>
+      </c>
+      <c r="D14" s="42" t="s">
+        <v>348</v>
+      </c>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42" t="s">
+        <v>370</v>
+      </c>
+      <c r="G14" s="42"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="42"/>
+      <c r="J14" s="42"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="42">
+        <v>4347.5</v>
+      </c>
+      <c r="B15" s="42" t="s">
+        <v>347</v>
+      </c>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42" t="s">
+        <v>349</v>
+      </c>
+      <c r="E15" s="42" t="s">
+        <v>244</v>
+      </c>
+      <c r="F15" s="42"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42" t="s">
+        <v>371</v>
+      </c>
+      <c r="I15" s="42"/>
+      <c r="J15" s="42"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="42">
+        <v>4625</v>
+      </c>
+      <c r="B16" s="42">
+        <v>100</v>
+      </c>
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="42"/>
+      <c r="J16" s="42"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="42">
+        <v>4768.8999999999996</v>
+      </c>
+      <c r="B17" s="42"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="42"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="42" t="s">
+        <v>372</v>
+      </c>
+      <c r="I17" s="42"/>
+      <c r="J17" s="42" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="42">
+        <v>4838</v>
+      </c>
+      <c r="B18" s="42" t="s">
+        <v>365</v>
+      </c>
+      <c r="C18" s="42"/>
+      <c r="D18" s="42" t="s">
+        <v>365</v>
+      </c>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="42"/>
+      <c r="J18" s="42"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="42">
+        <v>4853</v>
+      </c>
+      <c r="B19" s="42"/>
+      <c r="C19" s="42">
+        <v>100</v>
+      </c>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="42"/>
+      <c r="I19" s="42"/>
+      <c r="J19" s="42"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="42">
+        <v>4880.8999999999996</v>
+      </c>
+      <c r="B20" s="42"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="42" t="s">
+        <v>374</v>
+      </c>
+      <c r="E20" s="42" t="s">
+        <v>271</v>
+      </c>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="42"/>
+      <c r="I20" s="42"/>
+      <c r="J20" s="42"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="42">
+        <v>5008</v>
+      </c>
+      <c r="B21" s="42">
+        <v>100</v>
+      </c>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="42"/>
+      <c r="I21" s="42"/>
+      <c r="J21" s="42"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="42">
+        <v>5163</v>
+      </c>
+      <c r="B22" s="42"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42" t="s">
+        <v>365</v>
+      </c>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42" t="s">
+        <v>375</v>
+      </c>
+      <c r="H22" s="42" t="s">
+        <v>376</v>
+      </c>
+      <c r="I22" s="42"/>
+      <c r="J22" s="42"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="42">
+        <v>5214</v>
+      </c>
+      <c r="B23" s="42">
+        <v>100</v>
+      </c>
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="42"/>
+      <c r="I23" s="42"/>
+      <c r="J23" s="42"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="42">
+        <v>5400</v>
+      </c>
+      <c r="B24" s="42"/>
+      <c r="C24" s="42" t="s">
+        <v>377</v>
+      </c>
+      <c r="D24" s="42"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="42" t="s">
+        <v>377</v>
+      </c>
+      <c r="G24" s="42"/>
+      <c r="H24" s="42"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="42">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="42">
+        <v>5587</v>
+      </c>
+      <c r="B25" s="42"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="42" t="s">
+        <v>378</v>
+      </c>
+      <c r="E25" s="42" t="s">
+        <v>376</v>
+      </c>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="42"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="42"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="42">
+        <v>5598</v>
+      </c>
+      <c r="B26" s="42" t="s">
+        <v>379</v>
+      </c>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42" t="s">
+        <v>380</v>
+      </c>
+      <c r="E26" s="42"/>
+      <c r="F26" s="42"/>
+      <c r="G26" s="42"/>
+      <c r="H26" s="42"/>
+      <c r="I26" s="42"/>
+      <c r="J26" s="42"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="42">
+        <v>5645</v>
+      </c>
+      <c r="B27" s="42"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="42"/>
+      <c r="F27" s="42"/>
+      <c r="G27" s="42"/>
+      <c r="H27" s="42">
+        <v>100</v>
+      </c>
+      <c r="I27" s="42"/>
+      <c r="J27" s="42"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="42">
+        <v>5651</v>
+      </c>
+      <c r="B28" s="42"/>
+      <c r="C28" s="42"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="42"/>
+      <c r="G28" s="42">
+        <v>100</v>
+      </c>
+      <c r="H28" s="42"/>
+      <c r="I28" s="42"/>
+      <c r="J28" s="42"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="42">
+        <v>5682</v>
+      </c>
+      <c r="B29" s="42"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="42"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="42"/>
+      <c r="H29" s="42"/>
+      <c r="I29" s="42">
+        <v>100</v>
+      </c>
+      <c r="J29" s="42"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="42">
+        <v>5754</v>
+      </c>
+      <c r="B30" s="42"/>
+      <c r="C30" s="42"/>
+      <c r="D30" s="42"/>
+      <c r="E30" s="42"/>
+      <c r="F30" s="42"/>
+      <c r="G30" s="42"/>
+      <c r="H30" s="42"/>
+      <c r="I30" s="42"/>
+      <c r="J30" s="42">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="42">
+        <v>5802</v>
+      </c>
+      <c r="B31" s="42">
+        <v>100</v>
+      </c>
+      <c r="C31" s="42"/>
+      <c r="D31" s="42"/>
+      <c r="E31" s="42"/>
+      <c r="F31" s="42"/>
+      <c r="G31" s="42"/>
+      <c r="H31" s="42"/>
+      <c r="I31" s="42"/>
+      <c r="J31" s="42"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="42">
+        <v>6102</v>
+      </c>
+      <c r="B32" s="42" t="s">
+        <v>240</v>
+      </c>
+      <c r="C32" s="42" t="s">
+        <v>264</v>
+      </c>
+      <c r="D32" s="42"/>
+      <c r="E32" s="42"/>
+      <c r="F32" s="42"/>
+      <c r="G32" s="42"/>
+      <c r="H32" s="42"/>
+      <c r="I32" s="42"/>
+      <c r="J32" s="42"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" s="42">
+        <v>6489</v>
+      </c>
+      <c r="B33" s="42">
+        <v>100</v>
+      </c>
+      <c r="C33" s="42"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="42"/>
+      <c r="F33" s="42"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Enhance AI instruction files with CSV/tabular data processing safeguards
- Add CSV/Tabular Data Processing sections to large_scale_data_entry_prompt.md and copilot-instructions.md
- Include critical AI weakness mitigation for column alignment and blank cell handling
- Specify mandatory verification protocols: explicit column mapping, blank cell counting, bidirectional verification
- Add concrete examples showing correct vs incorrect column mapping approaches
- Update FRIBND.chatmode.md with communication guidelines: concise responses and meticulous attention to detail
- Minor updates to 1972HU10.ens and resonance branching ratios CSV for nuclear data processing
</commit_message>
<xml_diff>
--- a/A35/Cl35/temp/34Spg35Cl.xlsx
+++ b/A35/Cl35/temp/34Spg35Cl.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\X\ND\ENSDF\A35\Cl35\temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAECE17A-76D3-4868-9DED-C8CA5B392324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F36C417-9885-411E-A59C-9291E9A411BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="6" xr2:uid="{C580B2C4-D120-4EC4-942B-ED4733C9AE26}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="386">
   <si>
     <t>No.</t>
   </si>
@@ -1208,6 +1208,12 @@
   </si>
   <si>
     <t>≤ 0.2</t>
+  </si>
+  <si>
+    <t>Eg</t>
+  </si>
+  <si>
+    <t>BR</t>
   </si>
 </sst>
 </file>
@@ -1295,7 +1301,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1413,6 +1419,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1436,13 +1445,13 @@
     <xdr:from>
       <xdr:col>17</xdr:col>
       <xdr:colOff>43011</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>311334</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>69681</xdr:colOff>
-      <xdr:row>51</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>69399</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -14626,41 +14635,15 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
-      <c r="N52" s="7">
-        <f>$M51-N2</f>
-        <v>8382</v>
-      </c>
-      <c r="O52" s="7"/>
-      <c r="P52" s="7">
-        <f>$M51-P2</f>
-        <v>6619.2</v>
-      </c>
-      <c r="Q52" s="7">
-        <f t="shared" ref="P52:Y52" si="5">$M51-Q2</f>
-        <v>5736.4</v>
-      </c>
-      <c r="R52" s="7">
-        <f t="shared" si="5"/>
-        <v>5688</v>
-      </c>
-      <c r="S52" s="7">
-        <f t="shared" si="5"/>
-        <v>5379.3</v>
-      </c>
-      <c r="T52" s="7"/>
-      <c r="U52" s="7">
-        <f t="shared" si="5"/>
-        <v>4464.1000000000004</v>
-      </c>
-      <c r="V52" s="7"/>
-      <c r="W52" s="7"/>
-      <c r="X52" s="7"/>
-      <c r="Y52" s="7">
-        <f t="shared" si="5"/>
-        <v>4271</v>
-      </c>
-      <c r="Z52" s="7"/>
-      <c r="AA52" s="7"/>
+      <c r="K52" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="L52" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="M52" s="13" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="53" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A53" s="40">
@@ -14707,6 +14690,65 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="M54" s="23" t="s">
+        <v>385</v>
+      </c>
+      <c r="N54" s="26">
+        <f>N20</f>
+        <v>80</v>
+      </c>
+      <c r="O54" s="26">
+        <f t="shared" ref="O54:AA54" si="5">O20</f>
+        <v>0</v>
+      </c>
+      <c r="P54" s="26">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="Q54" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R54" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="S54" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T54" s="26">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="U54" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="V54" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="W54" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="X54" s="26">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="Y54" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Z54" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AA54" s="26">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
     </row>
     <row r="55" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A55" s="40">
@@ -14730,6 +14772,65 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="M55" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="N55" s="43">
+        <f>$M20-N2</f>
+        <v>7616</v>
+      </c>
+      <c r="O55" s="43">
+        <f>$M20-O2</f>
+        <v>6396.9</v>
+      </c>
+      <c r="P55" s="43">
+        <f>$M20-P2</f>
+        <v>5853.2</v>
+      </c>
+      <c r="Q55" s="43">
+        <f>$M20-Q2</f>
+        <v>4970.3999999999996</v>
+      </c>
+      <c r="R55" s="43">
+        <f>$M20-R2</f>
+        <v>4922</v>
+      </c>
+      <c r="S55" s="43">
+        <f>$M20-S2</f>
+        <v>4613.3</v>
+      </c>
+      <c r="T55" s="43">
+        <f>$M20-T2</f>
+        <v>4453.5</v>
+      </c>
+      <c r="U55" s="43">
+        <f>$M20-U2</f>
+        <v>3698.1</v>
+      </c>
+      <c r="V55" s="43">
+        <f>$M20-V2</f>
+        <v>3673.4</v>
+      </c>
+      <c r="W55" s="43">
+        <f>$M20-W2</f>
+        <v>3648.7</v>
+      </c>
+      <c r="X55" s="43">
+        <f>$M20-X2</f>
+        <v>3557.6</v>
+      </c>
+      <c r="Y55" s="43">
+        <f>$M20-Y2</f>
+        <v>3505</v>
+      </c>
+      <c r="Z55" s="43">
+        <f>$M20-Z2</f>
+        <v>3443</v>
+      </c>
+      <c r="AA55" s="43">
+        <f>$M20-AA2</f>
+        <v>3438.8</v>
+      </c>
     </row>
     <row r="56" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A56" s="40">
@@ -14753,6 +14854,62 @@
         <f t="shared" si="2"/>
         <v>0.3</v>
       </c>
+      <c r="N56" s="23" t="str">
+        <f>N1</f>
+        <v>Exf</v>
+      </c>
+      <c r="O56" s="23" t="str">
+        <f>O1</f>
+        <v>Exf</v>
+      </c>
+      <c r="P56" s="23" t="str">
+        <f>P1</f>
+        <v>Exf</v>
+      </c>
+      <c r="Q56" s="23" t="str">
+        <f>Q1</f>
+        <v>Exf</v>
+      </c>
+      <c r="R56" s="23" t="str">
+        <f>R1</f>
+        <v>Exf</v>
+      </c>
+      <c r="S56" s="23" t="str">
+        <f>S1</f>
+        <v>Exf</v>
+      </c>
+      <c r="T56" s="23" t="str">
+        <f>T1</f>
+        <v>Exf</v>
+      </c>
+      <c r="U56" s="23" t="str">
+        <f>U1</f>
+        <v>Exf</v>
+      </c>
+      <c r="V56" s="23" t="str">
+        <f>V1</f>
+        <v>Exf</v>
+      </c>
+      <c r="W56" s="23" t="str">
+        <f>W1</f>
+        <v>Exf</v>
+      </c>
+      <c r="X56" s="23" t="str">
+        <f>X1</f>
+        <v>Exf</v>
+      </c>
+      <c r="Y56" s="23" t="str">
+        <f>Y1</f>
+        <v>Exf</v>
+      </c>
+      <c r="Z56" s="23" t="str">
+        <f>Z1</f>
+        <v>Exf</v>
+      </c>
+      <c r="AA56" s="23" t="str">
+        <f>AA1</f>
+        <v>Exf</v>
+      </c>
     </row>
     <row r="57" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A57" s="40">
@@ -14775,6 +14932,62 @@
       <c r="F57" s="25">
         <f t="shared" si="2"/>
         <v>0.3</v>
+      </c>
+      <c r="N57" s="23">
+        <f>N2</f>
+        <v>0</v>
+      </c>
+      <c r="O57" s="23">
+        <f>O2</f>
+        <v>1219.0999999999999</v>
+      </c>
+      <c r="P57" s="23">
+        <f>P2</f>
+        <v>1762.8</v>
+      </c>
+      <c r="Q57" s="23">
+        <f>Q2</f>
+        <v>2645.6</v>
+      </c>
+      <c r="R57" s="23">
+        <f>R2</f>
+        <v>2694</v>
+      </c>
+      <c r="S57" s="23">
+        <f>S2</f>
+        <v>3002.7</v>
+      </c>
+      <c r="T57" s="23">
+        <f>T2</f>
+        <v>3162.5</v>
+      </c>
+      <c r="U57" s="23">
+        <f>U2</f>
+        <v>3917.9</v>
+      </c>
+      <c r="V57" s="23">
+        <f>V2</f>
+        <v>3942.6</v>
+      </c>
+      <c r="W57" s="23">
+        <f>W2</f>
+        <v>3967.3</v>
+      </c>
+      <c r="X57" s="23">
+        <f>X2</f>
+        <v>4058.4</v>
+      </c>
+      <c r="Y57" s="23">
+        <f>Y2</f>
+        <v>4111</v>
+      </c>
+      <c r="Z57" s="23">
+        <f>Z2</f>
+        <v>4173</v>
+      </c>
+      <c r="AA57" s="23">
+        <f>AA2</f>
+        <v>4177.2</v>
       </c>
     </row>
     <row r="58" spans="1:28" x14ac:dyDescent="0.2">

</xml_diff>